<commit_message>
Added Documents popup button
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -397,7 +397,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
@@ -452,12 +452,12 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -466,9 +466,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -791,36 +788,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="21"/>
+      <c r="B2" s="20"/>
       <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="21"/>
+      <c r="G2" s="20"/>
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -879,23 +876,23 @@
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
@@ -959,7 +956,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="22"/>
-      <c r="C9" s="25"/>
+      <c r="C9" s="12"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -974,23 +971,23 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
-      <c r="O10" s="20"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
@@ -1020,30 +1017,30 @@
       <c r="O11" s="19"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="21"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="21"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="20"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="21"/>
+      <c r="K12" s="20"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="21" t="s">
+      <c r="M12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="N12" s="21"/>
+      <c r="N12" s="20"/>
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1172,23 +1169,23 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="str">
@@ -1223,30 +1220,30 @@
       <c r="O19" s="19"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="21"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="21"/>
+      <c r="E20" s="20"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="21" t="s">
+      <c r="G20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="21"/>
+      <c r="H20" s="20"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="21" t="s">
+      <c r="J20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="K20" s="21"/>
+      <c r="K20" s="20"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="21"/>
+      <c r="N20" s="20"/>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1305,16 +1302,52 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J17:K17"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
@@ -1331,52 +1364,16 @@
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Insertion of islandr logo in home page and other minor changes
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -452,11 +452,11 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -777,47 +777,49 @@
   <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="10.7109375" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="8" width="10.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" customWidth="1"/>
+    <col min="10" max="11" width="10.7109375" customWidth="1"/>
     <col min="12" max="12" width="15.7109375" customWidth="1"/>
-    <col min="14" max="14" width="10.28515625" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" customWidth="1"/>
     <col min="15" max="15" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="20"/>
+      <c r="L1" s="20"/>
+      <c r="M1" s="20"/>
+      <c r="N1" s="20"/>
+      <c r="O1" s="20"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="21"/>
       <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="20"/>
+      <c r="G2" s="21"/>
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -876,23 +878,23 @@
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="21"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
@@ -971,23 +973,23 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
+      <c r="K10" s="20"/>
+      <c r="L10" s="20"/>
+      <c r="M10" s="20"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="20"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
@@ -1017,30 +1019,30 @@
       <c r="O11" s="19"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="20"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="20"/>
+      <c r="E12" s="21"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="20"/>
+      <c r="H12" s="21"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="20"/>
+      <c r="K12" s="21"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="20" t="s">
+      <c r="M12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="N12" s="20"/>
+      <c r="N12" s="21"/>
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1169,23 +1171,23 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="20"/>
+      <c r="K18" s="20"/>
+      <c r="L18" s="20"/>
+      <c r="M18" s="20"/>
+      <c r="N18" s="20"/>
+      <c r="O18" s="20"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="str">
@@ -1220,30 +1222,30 @@
       <c r="O19" s="19"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="20"/>
+      <c r="B20" s="21"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="20"/>
+      <c r="E20" s="21"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="20"/>
+      <c r="H20" s="21"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="K20" s="20"/>
+      <c r="K20" s="21"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="20" t="s">
+      <c r="M20" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="20"/>
+      <c r="N20" s="21"/>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1302,6 +1304,62 @@
     </row>
   </sheetData>
   <mergeCells count="72">
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A5:O5"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -1318,62 +1376,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Implementation of vertical navbar's buttons colour change when Frame is active
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>Soil</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>Coordinates (lat-lng)</t>
+  </si>
+  <si>
+    <t>Site Area [km²]</t>
   </si>
 </sst>
 </file>
@@ -397,7 +400,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
@@ -452,12 +455,12 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -465,6 +468,12 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -790,36 +799,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="21"/>
+      <c r="B2" s="20"/>
       <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="G2" s="21"/>
+      <c r="G2" s="20"/>
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -877,47 +886,47 @@
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
-    <row r="5" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="26"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
-      <c r="J5" s="20"/>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="22"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="2"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="4"/>
@@ -936,7 +945,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8" s="22"/>
       <c r="C8" s="4"/>
@@ -973,23 +982,23 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-      <c r="K10" s="20"/>
-      <c r="L10" s="20"/>
-      <c r="M10" s="20"/>
-      <c r="N10" s="20"/>
-      <c r="O10" s="20"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
@@ -1019,30 +1028,30 @@
       <c r="O11" s="19"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="21"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="21" t="s">
+      <c r="D12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="21"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="21" t="s">
+      <c r="G12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="21"/>
+      <c r="H12" s="20"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="21" t="s">
+      <c r="J12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="21"/>
+      <c r="K12" s="20"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="21" t="s">
+      <c r="M12" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="N12" s="21"/>
+      <c r="N12" s="20"/>
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1171,23 +1180,23 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="str">
@@ -1222,30 +1231,30 @@
       <c r="O19" s="19"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="21"/>
+      <c r="B20" s="20"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="21" t="s">
+      <c r="D20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="21"/>
+      <c r="E20" s="20"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="21" t="s">
+      <c r="G20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="21"/>
+      <c r="H20" s="20"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="21" t="s">
+      <c r="J20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="K20" s="21"/>
+      <c r="K20" s="20"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="21" t="s">
+      <c r="M20" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="21"/>
+      <c r="N20" s="20"/>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1303,17 +1312,55 @@
       <c r="O22" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="72">
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
+  <mergeCells count="74">
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="J17:K17"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
@@ -1330,52 +1377,16 @@
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A5:O5"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Implementation of 3 scenarios reporting
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -4,10 +4,12 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="On-site on-site" sheetId="3" r:id="rId1"/>
+    <sheet name="On-site off-site" sheetId="2" r:id="rId2"/>
+    <sheet name="Off-site on-site" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="41">
   <si>
     <t>Soil</t>
   </si>
@@ -116,9 +118,6 @@
     <t>Source</t>
   </si>
   <si>
-    <t>Summary</t>
-  </si>
-  <si>
     <t>Assessment date</t>
   </si>
   <si>
@@ -144,6 +143,15 @@
   </si>
   <si>
     <t>Site Area [km²]</t>
+  </si>
+  <si>
+    <t>Summary (On-site to on-site contamination)</t>
+  </si>
+  <si>
+    <t>Summary (On-site to off-site contamination)</t>
+  </si>
+  <si>
+    <t>Summary (Off-site to on-site contamination)</t>
   </si>
 </sst>
 </file>
@@ -446,6 +454,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -455,25 +469,19 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -799,64 +807,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="A1" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="20"/>
+      <c r="B2" s="17"/>
       <c r="C2" s="3"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="20"/>
+      <c r="F2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="17"/>
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="L2" s="24"/>
+      <c r="K2" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="26"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B3" s="16"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L3" s="16"/>
       <c r="M3" s="9"/>
@@ -865,21 +873,21 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="23"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="1"/>
       <c r="F4" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G4" s="23"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="L4" s="23"/>
       <c r="M4" s="9"/>
@@ -887,42 +895,42 @@
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="26"/>
+      <c r="A5" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="25"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="26"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="26"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="22" t="s">
@@ -982,76 +990,76 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="17" t="s">
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="17" t="s">
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="17" t="s">
+      <c r="H11" s="20"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="18"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="17" t="s">
+      <c r="K11" s="20"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="N11" s="18"/>
-      <c r="O11" s="19"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="21"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="20"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="20"/>
+      <c r="E12" s="17"/>
       <c r="F12" s="4"/>
-      <c r="G12" s="20" t="s">
+      <c r="G12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="20"/>
+      <c r="H12" s="17"/>
       <c r="I12" s="4"/>
-      <c r="J12" s="20" t="s">
+      <c r="J12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="K12" s="20"/>
+      <c r="K12" s="17"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="20" t="s">
+      <c r="M12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="N12" s="20"/>
+      <c r="N12" s="17"/>
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
@@ -1180,81 +1188,81 @@
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="str">
+      <c r="A19" s="19" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="18"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="17" t="str">
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="19" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="18"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="17" t="str">
+      <c r="E19" s="20"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="19" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="18"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="17" t="str">
+      <c r="H19" s="20"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="19" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="18"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="17" t="str">
+      <c r="K19" s="20"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="19" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="18"/>
-      <c r="O19" s="19"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="21"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B20" s="20"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="E20" s="20"/>
+      <c r="E20" s="17"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="H20" s="20"/>
+      <c r="H20" s="17"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="20" t="s">
+      <c r="J20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="K20" s="20"/>
+      <c r="K20" s="17"/>
       <c r="L20" s="4"/>
-      <c r="M20" s="20" t="s">
+      <c r="M20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="N20" s="20"/>
+      <c r="N20" s="17"/>
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1313,8 +1321,1230 @@
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="17"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="26"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="16"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="16"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="23"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="23"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="20"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="N11" s="20"/>
+      <c r="O11" s="21"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="K12" s="17"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="N12" s="17"/>
+      <c r="O12" s="7"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="16"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="16"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N13" s="16"/>
+      <c r="O13" s="7"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="16"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" s="16"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="N14" s="16"/>
+      <c r="O14" s="7"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="16"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N15" s="16"/>
+      <c r="O15" s="7"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="8"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="16"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="K17" s="16"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="N17" s="16"/>
+      <c r="O17" s="14"/>
+    </row>
+    <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="str">
+        <f>A11</f>
+        <v>Soil</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="19" t="str">
+        <f t="shared" ref="D19" si="0">D11</f>
+        <v>Ground water</v>
+      </c>
+      <c r="E19" s="20"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="19" t="str">
+        <f t="shared" ref="G19" si="1">G11</f>
+        <v>Surface water</v>
+      </c>
+      <c r="H19" s="20"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="19" t="str">
+        <f t="shared" ref="J19" si="2">J11</f>
+        <v>Air</v>
+      </c>
+      <c r="K19" s="20"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="19" t="str">
+        <f t="shared" ref="M19" si="3">M11</f>
+        <v>Sediment</v>
+      </c>
+      <c r="N19" s="20"/>
+      <c r="O19" s="21"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="17"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" s="17"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="N20" s="17"/>
+      <c r="O20" s="7"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" s="16"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21" s="16"/>
+      <c r="O21" s="7"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="16"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="16"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="K22" s="16"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="16"/>
+      <c r="O22" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="74">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:O22"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="10.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
+    <col min="7" max="8" width="10.7109375" customWidth="1"/>
+    <col min="9" max="9" width="15.7109375" customWidth="1"/>
+    <col min="10" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" customWidth="1"/>
+    <col min="13" max="14" width="10.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+      <c r="M1" s="18"/>
+      <c r="N1" s="18"/>
+      <c r="O1" s="18"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="17"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="26"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="16"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="16"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="23"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" s="23"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A6" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="18"/>
+      <c r="N6" s="18"/>
+      <c r="O6" s="18"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="22"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="22"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
+      <c r="N10" s="18"/>
+      <c r="O10" s="18"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="19" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="H11" s="20"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" s="20"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="N11" s="20"/>
+      <c r="O11" s="21"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="17"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="K12" s="17"/>
+      <c r="L12" s="4"/>
+      <c r="M12" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="N12" s="17"/>
+      <c r="O12" s="7"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="16"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="16"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="16"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="16"/>
+      <c r="L13" s="4"/>
+      <c r="M13" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N13" s="16"/>
+      <c r="O13" s="7"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="16"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="16"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="K14" s="16"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="N14" s="16"/>
+      <c r="O14" s="7"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="K15" s="16"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="N15" s="16"/>
+      <c r="O15" s="7"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="8"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="E17" s="16"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" s="16"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="K17" s="16"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="N17" s="16"/>
+      <c r="O17" s="14"/>
+    </row>
+    <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
+      <c r="A18" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="18"/>
+      <c r="M18" s="18"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="18"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="19" t="str">
+        <f>A11</f>
+        <v>Soil</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="19" t="str">
+        <f t="shared" ref="D19" si="0">D11</f>
+        <v>Ground water</v>
+      </c>
+      <c r="E19" s="20"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="19" t="str">
+        <f t="shared" ref="G19" si="1">G11</f>
+        <v>Surface water</v>
+      </c>
+      <c r="H19" s="20"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="19" t="str">
+        <f t="shared" ref="J19" si="2">J11</f>
+        <v>Air</v>
+      </c>
+      <c r="K19" s="20"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="19" t="str">
+        <f t="shared" ref="M19" si="3">M11</f>
+        <v>Sediment</v>
+      </c>
+      <c r="N19" s="20"/>
+      <c r="O19" s="21"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="17"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" s="17"/>
+      <c r="L20" s="4"/>
+      <c r="M20" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="N20" s="17"/>
+      <c r="O20" s="7"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H21" s="16"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="K21" s="16"/>
+      <c r="L21" s="4"/>
+      <c r="M21" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="N21" s="16"/>
+      <c r="O21" s="7"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="16"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="16"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="16"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="K22" s="16"/>
+      <c r="L22" s="11"/>
+      <c r="M22" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="16"/>
+      <c r="O22" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="74">
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -1329,8 +2559,8 @@
     <mergeCell ref="G17:H17"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A6:O6"/>
     <mergeCell ref="A8:B8"/>
@@ -1345,35 +2575,35 @@
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="K3:L3"/>
     <mergeCell ref="K4:L4"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="M13:N13"/>
     <mergeCell ref="M14:N14"/>
     <mergeCell ref="M15:N15"/>
-    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="J12:K12"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J15:K15"/>
-    <mergeCell ref="J17:K17"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A21:B21"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
     <mergeCell ref="M22:N22"/>
     <mergeCell ref="G20:H20"/>
     <mergeCell ref="G21:H21"/>
@@ -1382,11 +2612,13 @@
     <mergeCell ref="J20:K20"/>
     <mergeCell ref="J21:K21"/>
     <mergeCell ref="J22:K22"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G15:H15"/>
     <mergeCell ref="G16:H16"/>
     <mergeCell ref="J16:K16"/>
     <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Saving pngs into excel
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" activeTab="2"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="On-site on-site" sheetId="3" r:id="rId1"/>
     <sheet name="On-site off-site" sheetId="2" r:id="rId2"/>
     <sheet name="Off-site on-site" sheetId="1" r:id="rId3"/>
+    <sheet name="pics" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="152511"/>
   <extLst>
@@ -451,14 +452,26 @@
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -471,18 +484,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -807,23 +808,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
@@ -840,103 +841,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="26"/>
+      <c r="L2" s="18"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="16"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="16"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="20"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="20"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="22"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -952,10 +953,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -971,10 +972,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="12"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -990,50 +991,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="19" t="s">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="19" t="s">
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="24"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="20"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="19" t="s">
+      <c r="K11" s="24"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="25"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
@@ -1063,180 +1064,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="16"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="16"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="16"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N13" s="16"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="16"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="16" t="s">
+      <c r="M14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N14" s="16"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="16"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="16"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="16" t="s">
+      <c r="M15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="N15" s="16"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="16"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H17" s="16"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="16" t="s">
+      <c r="J17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="16"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="16" t="s">
+      <c r="M17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="N17" s="16"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="str">
+      <c r="A19" s="23" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="19" t="str">
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="23" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="19" t="str">
+      <c r="E19" s="24"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="23" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="19" t="str">
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="23" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="20"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="19" t="str">
+      <c r="K19" s="24"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="23" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="20"/>
-      <c r="O19" s="21"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
@@ -1266,61 +1267,128 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="16"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="16"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="16" t="s">
+      <c r="J21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="16" t="s">
+      <c r="M21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="N21" s="16"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="11"/>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="16"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="11"/>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="16" t="s">
+      <c r="J22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="K22" s="16"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="11"/>
-      <c r="M22" s="16" t="s">
+      <c r="M22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="N22" s="16"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -1328,73 +1396,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1419,23 +1420,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
@@ -1452,103 +1453,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="26"/>
+      <c r="L2" s="18"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="16"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="16"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="20"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="20"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="22"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1564,10 +1565,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1583,10 +1584,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="12"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1602,50 +1603,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="19" t="s">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="19" t="s">
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="24"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="20"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="19" t="s">
+      <c r="K11" s="24"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="25"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
@@ -1675,180 +1676,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="16"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="16"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="16"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N13" s="16"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="16"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="16" t="s">
+      <c r="M14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N14" s="16"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="16"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="16"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="16" t="s">
+      <c r="M15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="N15" s="16"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="16"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H17" s="16"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="16" t="s">
+      <c r="J17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="16"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="16" t="s">
+      <c r="M17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="N17" s="16"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="str">
+      <c r="A19" s="23" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="19" t="str">
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="23" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="19" t="str">
+      <c r="E19" s="24"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="23" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="19" t="str">
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="23" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="20"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="19" t="str">
+      <c r="K19" s="24"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="23" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="20"/>
-      <c r="O19" s="21"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
@@ -1878,61 +1879,128 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="16"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="16"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="16" t="s">
+      <c r="J21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="16" t="s">
+      <c r="M21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="N21" s="16"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="11"/>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="16"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="11"/>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="16" t="s">
+      <c r="J22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="K22" s="16"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="11"/>
-      <c r="M22" s="16" t="s">
+      <c r="M22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="N22" s="16"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -1940,73 +2008,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2031,23 +2032,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="16"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
@@ -2064,103 +2065,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="26" t="s">
+      <c r="K2" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="26"/>
+      <c r="L2" s="18"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="16"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="16"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="16" t="s">
+      <c r="K3" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="16"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="20"/>
       <c r="C4" s="15"/>
       <c r="D4" s="15"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="20"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="20"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="22"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="22"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="18" t="s">
+      <c r="A6" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="22"/>
+      <c r="B7" s="26"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -2176,10 +2177,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="22"/>
+      <c r="B8" s="26"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2195,10 +2196,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="22"/>
+      <c r="B9" s="26"/>
       <c r="C9" s="12"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -2214,50 +2215,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="19" t="s">
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="19" t="s">
+      <c r="E11" s="24"/>
+      <c r="F11" s="25"/>
+      <c r="G11" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="19" t="s">
+      <c r="H11" s="24"/>
+      <c r="I11" s="25"/>
+      <c r="J11" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="K11" s="20"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="19" t="s">
+      <c r="K11" s="24"/>
+      <c r="L11" s="25"/>
+      <c r="M11" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="N11" s="20"/>
-      <c r="O11" s="21"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="25"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
@@ -2287,180 +2288,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="16" t="s">
+      <c r="D13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="16"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="16"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="16"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N13" s="16"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="16" t="s">
+      <c r="D14" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="16"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="16" t="s">
+      <c r="G14" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="16"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="16" t="s">
+      <c r="J14" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K14" s="16"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="16" t="s">
+      <c r="M14" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N14" s="16"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="16"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="16" t="s">
+      <c r="J15" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="K15" s="16"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="16" t="s">
+      <c r="M15" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="N15" s="16"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="16"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="16"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="16"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="12"/>
-      <c r="D17" s="16" t="s">
+      <c r="D17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="16" t="s">
+      <c r="G17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="H17" s="16"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="16" t="s">
+      <c r="J17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="16"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="16" t="s">
+      <c r="M17" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="N17" s="16"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="14"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="str">
+      <c r="A19" s="23" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="20"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="19" t="str">
+      <c r="B19" s="24"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="23" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="20"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="19" t="str">
+      <c r="E19" s="24"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="23" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="19" t="str">
+      <c r="H19" s="24"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="23" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="20"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="19" t="str">
+      <c r="K19" s="24"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="23" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="20"/>
-      <c r="O19" s="21"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="25"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
@@ -2490,61 +2491,119 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="16"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="16" t="s">
+      <c r="G21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="H21" s="16"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="16" t="s">
+      <c r="J21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="16"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="16" t="s">
+      <c r="M21" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="N21" s="16"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="11"/>
-      <c r="D22" s="16" t="s">
+      <c r="D22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E22" s="16"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="11"/>
-      <c r="G22" s="16" t="s">
+      <c r="G22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="H22" s="16"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="16" t="s">
+      <c r="J22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="K22" s="16"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="11"/>
-      <c r="M22" s="16" t="s">
+      <c r="M22" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="N22" s="16"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -2561,66 +2620,17 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: :construction: Change report to address CRS implementation
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" activeTab="4"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
   </bookViews>
   <sheets>
     <sheet name="On-site on-site" sheetId="3" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="48">
   <si>
     <t>Soil</t>
   </si>
@@ -172,6 +172,9 @@
   </si>
   <si>
     <t>Name</t>
+  </si>
+  <si>
+    <t>CRS type</t>
   </si>
 </sst>
 </file>
@@ -471,26 +474,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -503,6 +494,18 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -828,23 +831,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -861,103 +864,105 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="29"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="22"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="22"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="22"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="23"/>
+      <c r="A4" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="26"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="26"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="25"/>
+      <c r="A5" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="28"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" s="28"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="28"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="25"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -973,10 +978,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -992,10 +997,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1011,50 +1016,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="26" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="26" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="26" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="27"/>
-      <c r="L11" s="28"/>
-      <c r="M11" s="26" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="27"/>
-      <c r="O11" s="28"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -1084,180 +1089,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="22"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="22"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="22"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="22"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="22"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="22" t="s">
+      <c r="J14" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="22"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="22"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="22"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="22" t="s">
+      <c r="J15" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="22"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="22" t="s">
+      <c r="M15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="22"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="22"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="22"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="22"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="22" t="s">
+      <c r="M17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="22"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="26" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="26" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="26" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="27"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="26" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="27"/>
-      <c r="O19" s="28"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -1287,128 +1292,61 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="22"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="22"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="22"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="22" t="s">
+      <c r="J21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="22"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="22" t="s">
+      <c r="M21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="22"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="22"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="22"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="22"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="22"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -1416,6 +1354,73 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1440,23 +1445,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -1473,103 +1478,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="29"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="22"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="22"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="22"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="26"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="26"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="28"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="28"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="28"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="25"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1585,10 +1590,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1604,10 +1609,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1623,50 +1628,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="26" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="26" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="26" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="27"/>
-      <c r="L11" s="28"/>
-      <c r="M11" s="26" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="27"/>
-      <c r="O11" s="28"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -1696,180 +1701,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="22"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="22"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="22"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="22"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="22"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="22" t="s">
+      <c r="J14" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="22"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="22"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="22"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="22" t="s">
+      <c r="J15" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="22"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="22" t="s">
+      <c r="M15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="22"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="22"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="22"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="22"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="22" t="s">
+      <c r="M17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="22"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="26" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="26" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="26" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="27"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="26" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="27"/>
-      <c r="O19" s="28"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -1899,128 +1904,61 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="22"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="22"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="22"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="22" t="s">
+      <c r="J21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="22"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="22" t="s">
+      <c r="M21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="22"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="22"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="22"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="22"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="22"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -2028,6 +1966,73 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2052,23 +2057,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -2085,103 +2090,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="21" t="s">
+      <c r="K2" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="21"/>
+      <c r="L2" s="29"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="22"/>
+      <c r="B3" s="19"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="22"/>
+      <c r="G3" s="19"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="22"/>
+      <c r="L3" s="19"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="26"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="23"/>
+      <c r="G4" s="26"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="23"/>
+      <c r="L4" s="26"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="25"/>
+      <c r="B5" s="28"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="25"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="28"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="24"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="27"/>
+      <c r="L5" s="28"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="19"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="25"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -2197,10 +2202,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2216,10 +2221,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="29" t="s">
+      <c r="A9" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -2235,50 +2240,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
-      <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
-      <c r="L10" s="19"/>
-      <c r="M10" s="19"/>
-      <c r="N10" s="19"/>
-      <c r="O10" s="19"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
+      <c r="A11" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="26" t="s">
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="27"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="26" t="s">
+      <c r="E11" s="23"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="27"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="26" t="s">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="27"/>
-      <c r="L11" s="28"/>
-      <c r="M11" s="26" t="s">
+      <c r="K11" s="23"/>
+      <c r="L11" s="24"/>
+      <c r="M11" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="27"/>
-      <c r="O11" s="28"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="24"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -2308,180 +2313,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="22"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="22"/>
+      <c r="E13" s="19"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="22"/>
+      <c r="H13" s="19"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="22"/>
+      <c r="K13" s="19"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="22"/>
+      <c r="N13" s="19"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="22"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="22"/>
+      <c r="E14" s="19"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="22"/>
+      <c r="H14" s="19"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="22" t="s">
+      <c r="J14" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="22"/>
+      <c r="K14" s="19"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="22"/>
+      <c r="N14" s="19"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="22"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="22"/>
+      <c r="E15" s="19"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="19"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="22" t="s">
+      <c r="J15" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="22"/>
+      <c r="K15" s="19"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="22" t="s">
+      <c r="M15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="22"/>
+      <c r="N15" s="19"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="22"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="G16" s="19"/>
+      <c r="H16" s="19"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="22"/>
+      <c r="E17" s="19"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="22" t="s">
+      <c r="G17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="22"/>
+      <c r="H17" s="19"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="22"/>
+      <c r="K17" s="19"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="22" t="s">
+      <c r="M17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="22"/>
+      <c r="N17" s="19"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="21"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="26" t="str">
+      <c r="A19" s="22" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="26" t="str">
+      <c r="B19" s="23"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="22" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="26" t="str">
+      <c r="E19" s="23"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="22" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="27"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="26" t="str">
+      <c r="H19" s="23"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="22" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="27"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="26" t="str">
+      <c r="K19" s="23"/>
+      <c r="L19" s="24"/>
+      <c r="M19" s="22" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="27"/>
-      <c r="O19" s="28"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="24"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -2511,103 +2516,77 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="22"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="22"/>
+      <c r="E21" s="19"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="22" t="s">
+      <c r="G21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="22"/>
+      <c r="H21" s="19"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="22" t="s">
+      <c r="J21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="22"/>
+      <c r="K21" s="19"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="22" t="s">
+      <c r="M21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="22"/>
+      <c r="N21" s="19"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="22"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="22"/>
+      <c r="E22" s="19"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="22"/>
+      <c r="H22" s="19"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="22" t="s">
+      <c r="J22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="22"/>
+      <c r="K22" s="19"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="22"/>
+      <c r="N22" s="19"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A6:O6"/>
     <mergeCell ref="A8:B8"/>
@@ -2624,22 +2603,48 @@
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: :sparkles: Add more CRS selections
</commit_message>
<xml_diff>
--- a/rss_islandr/templates/report_template.xlsx
+++ b/rss_islandr/templates/report_template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11385" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="On-site on-site" sheetId="3" r:id="rId1"/>
@@ -474,14 +474,26 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="3" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -494,18 +506,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="4" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -831,23 +831,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -864,105 +864,105 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="29"/>
+      <c r="L2" s="21"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="19"/>
+      <c r="L3" s="22"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="26"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="26"/>
+      <c r="G4" s="23"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="26" t="s">
+      <c r="K4" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="26"/>
+      <c r="L4" s="23"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="28"/>
+      <c r="B5" s="25"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="28"/>
+      <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="28"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -978,10 +978,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -997,10 +997,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="25"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1016,50 +1016,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22" t="s">
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="22" t="s">
+      <c r="K11" s="27"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="24"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="28"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -1089,180 +1089,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="19"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="19"/>
+      <c r="H13" s="22"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="19"/>
+      <c r="K13" s="22"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="19" t="s">
+      <c r="M13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="19"/>
+      <c r="N13" s="22"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="19"/>
+      <c r="B14" s="22"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="19"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="19"/>
+      <c r="H14" s="22"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="19"/>
+      <c r="K14" s="22"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="19"/>
+      <c r="N14" s="22"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="19"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="19"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="19" t="s">
+      <c r="J15" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="19"/>
+      <c r="K15" s="22"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="19"/>
+      <c r="N15" s="22"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="19"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="19"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="19"/>
+      <c r="H17" s="22"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="19" t="s">
+      <c r="J17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="19"/>
+      <c r="K17" s="22"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="19" t="s">
+      <c r="M17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="19"/>
+      <c r="N17" s="22"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="str">
+      <c r="A19" s="26" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="22" t="str">
+      <c r="B19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="26" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22" t="str">
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="26" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22" t="str">
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="26" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="22" t="str">
+      <c r="K19" s="27"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="26" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="23"/>
-      <c r="O19" s="24"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="28"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -1292,61 +1292,128 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="19"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="19"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="19"/>
+      <c r="H21" s="22"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="22"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="19" t="s">
+      <c r="M21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="19"/>
+      <c r="N21" s="22"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="19"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="19"/>
+      <c r="H22" s="22"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="19"/>
+      <c r="K22" s="22"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="19" t="s">
+      <c r="M22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="19"/>
+      <c r="N22" s="22"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -1354,73 +1421,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -1445,23 +1445,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -1478,103 +1478,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="29"/>
+      <c r="L2" s="21"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="19"/>
+      <c r="L3" s="22"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="26"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="26"/>
+      <c r="G4" s="23"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="26" t="s">
+      <c r="K4" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="26"/>
+      <c r="L4" s="23"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="28"/>
+      <c r="B5" s="25"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="28"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="28"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1590,10 +1590,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1609,10 +1609,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="25"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1628,50 +1628,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22" t="s">
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="22" t="s">
+      <c r="K11" s="27"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="24"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="28"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -1701,180 +1701,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="19"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="19"/>
+      <c r="H13" s="22"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="19"/>
+      <c r="K13" s="22"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="19" t="s">
+      <c r="M13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="19"/>
+      <c r="N13" s="22"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="19"/>
+      <c r="B14" s="22"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="19"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="19"/>
+      <c r="H14" s="22"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="19"/>
+      <c r="K14" s="22"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="19"/>
+      <c r="N14" s="22"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="19"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="19"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="19" t="s">
+      <c r="J15" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="19"/>
+      <c r="K15" s="22"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="19"/>
+      <c r="N15" s="22"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="19"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="19"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="19"/>
+      <c r="H17" s="22"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="19" t="s">
+      <c r="J17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="19"/>
+      <c r="K17" s="22"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="19" t="s">
+      <c r="M17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="19"/>
+      <c r="N17" s="22"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="str">
+      <c r="A19" s="26" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="22" t="str">
+      <c r="B19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="26" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22" t="str">
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="26" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22" t="str">
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="26" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="22" t="str">
+      <c r="K19" s="27"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="26" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="23"/>
-      <c r="O19" s="24"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="28"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -1904,61 +1904,128 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="19"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="19"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="19"/>
+      <c r="H21" s="22"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="22"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="19" t="s">
+      <c r="M21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="19"/>
+      <c r="N21" s="22"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="19"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="19"/>
+      <c r="H22" s="22"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="19"/>
+      <c r="K22" s="22"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="19" t="s">
+      <c r="M22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="19"/>
+      <c r="N22" s="22"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:O10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="J11:L11"/>
+    <mergeCell ref="M11:O11"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="K5:L5"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="F2:G2"/>
@@ -1966,73 +2033,6 @@
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="K3:L3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="J11:L11"/>
-    <mergeCell ref="M11:O11"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:O10"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2057,23 +2057,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
@@ -2090,103 +2090,103 @@
       <c r="H2" s="3"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="29" t="s">
+      <c r="K2" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="29"/>
+      <c r="L2" s="21"/>
       <c r="M2" s="3"/>
       <c r="N2" s="1"/>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="19"/>
+      <c r="B3" s="22"/>
       <c r="C3" s="9"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G3" s="19"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="3"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="19"/>
+      <c r="L3" s="22"/>
       <c r="M3" s="9"/>
       <c r="N3" s="1"/>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="26"/>
+      <c r="B4" s="23"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="1"/>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="26"/>
+      <c r="G4" s="23"/>
       <c r="H4" s="3"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
-      <c r="K4" s="26" t="s">
+      <c r="K4" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="L4" s="26"/>
+      <c r="L4" s="23"/>
       <c r="M4" s="9"/>
       <c r="N4" s="1"/>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="28"/>
+      <c r="B5" s="25"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10"/>
       <c r="E5" s="1"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="28"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="25"/>
       <c r="H5" s="3"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="28"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
       <c r="M5" s="9"/>
       <c r="N5" s="1"/>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="25"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -2202,10 +2202,10 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="25"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -2221,10 +2221,10 @@
       <c r="O8" s="2"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="25"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="13"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -2240,50 +2240,50 @@
       <c r="O9" s="2"/>
     </row>
     <row r="10" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="22" t="s">
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="23"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22" t="s">
+      <c r="E11" s="27"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="H11" s="23"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="22" t="s">
+      <c r="H11" s="27"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="23"/>
-      <c r="L11" s="24"/>
-      <c r="M11" s="22" t="s">
+      <c r="K11" s="27"/>
+      <c r="L11" s="28"/>
+      <c r="M11" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="N11" s="23"/>
-      <c r="O11" s="24"/>
+      <c r="N11" s="27"/>
+      <c r="O11" s="28"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
@@ -2313,180 +2313,180 @@
       <c r="O12" s="7"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="19"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="19"/>
+      <c r="E13" s="22"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="19"/>
+      <c r="H13" s="22"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="19" t="s">
+      <c r="J13" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="19"/>
+      <c r="K13" s="22"/>
       <c r="L13" s="4"/>
-      <c r="M13" s="19" t="s">
+      <c r="M13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="N13" s="19"/>
+      <c r="N13" s="22"/>
       <c r="O13" s="7"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="A14" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="19"/>
+      <c r="B14" s="22"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="E14" s="19"/>
+      <c r="E14" s="22"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="19"/>
+      <c r="H14" s="22"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="19" t="s">
+      <c r="J14" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="K14" s="19"/>
+      <c r="K14" s="22"/>
       <c r="L14" s="4"/>
-      <c r="M14" s="19" t="s">
+      <c r="M14" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="N14" s="19"/>
+      <c r="N14" s="22"/>
       <c r="O14" s="7"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="19"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="19" t="s">
+      <c r="D15" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="19"/>
+      <c r="E15" s="22"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="19" t="s">
+      <c r="J15" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="19"/>
+      <c r="K15" s="22"/>
       <c r="L15" s="4"/>
-      <c r="M15" s="19" t="s">
+      <c r="M15" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="N15" s="19"/>
+      <c r="N15" s="22"/>
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
+      <c r="A16" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="19"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
       <c r="I16" s="6"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
       <c r="L16" s="5"/>
-      <c r="M16" s="19"/>
-      <c r="N16" s="19"/>
+      <c r="M16" s="22"/>
+      <c r="N16" s="22"/>
       <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="19"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="13"/>
-      <c r="D17" s="19" t="s">
+      <c r="D17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="19"/>
+      <c r="E17" s="22"/>
       <c r="F17" s="13"/>
-      <c r="G17" s="19" t="s">
+      <c r="G17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="H17" s="19"/>
+      <c r="H17" s="22"/>
       <c r="I17" s="13"/>
-      <c r="J17" s="19" t="s">
+      <c r="J17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="K17" s="19"/>
+      <c r="K17" s="22"/>
       <c r="L17" s="13"/>
-      <c r="M17" s="19" t="s">
+      <c r="M17" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="19"/>
+      <c r="N17" s="22"/>
       <c r="O17" s="13"/>
     </row>
     <row r="18" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
-      <c r="H18" s="21"/>
-      <c r="I18" s="21"/>
-      <c r="J18" s="21"/>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="21"/>
-      <c r="O18" s="21"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="19"/>
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="str">
+      <c r="A19" s="26" t="str">
         <f>A11</f>
         <v>Soil</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="22" t="str">
+      <c r="B19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="26" t="str">
         <f t="shared" ref="D19" si="0">D11</f>
         <v>Ground water</v>
       </c>
-      <c r="E19" s="23"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="22" t="str">
+      <c r="E19" s="27"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="26" t="str">
         <f t="shared" ref="G19" si="1">G11</f>
         <v>Surface water</v>
       </c>
-      <c r="H19" s="23"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="22" t="str">
+      <c r="H19" s="27"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="26" t="str">
         <f t="shared" ref="J19" si="2">J11</f>
         <v>Air</v>
       </c>
-      <c r="K19" s="23"/>
-      <c r="L19" s="24"/>
-      <c r="M19" s="22" t="str">
+      <c r="K19" s="27"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="26" t="str">
         <f t="shared" ref="M19" si="3">M11</f>
         <v>Sediment</v>
       </c>
-      <c r="N19" s="23"/>
-      <c r="O19" s="24"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="28"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="20" t="s">
@@ -2516,61 +2516,119 @@
       <c r="O20" s="7"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="19"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="19" t="s">
+      <c r="D21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="E21" s="19"/>
+      <c r="E21" s="22"/>
       <c r="F21" s="4"/>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="H21" s="19"/>
+      <c r="H21" s="22"/>
       <c r="I21" s="4"/>
-      <c r="J21" s="19" t="s">
+      <c r="J21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="K21" s="19"/>
+      <c r="K21" s="22"/>
       <c r="L21" s="4"/>
-      <c r="M21" s="19" t="s">
+      <c r="M21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="N21" s="19"/>
+      <c r="N21" s="22"/>
       <c r="O21" s="7"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="13"/>
-      <c r="D22" s="19" t="s">
+      <c r="D22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E22" s="19"/>
+      <c r="E22" s="22"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H22" s="19"/>
+      <c r="H22" s="22"/>
       <c r="I22" s="13"/>
-      <c r="J22" s="19" t="s">
+      <c r="J22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="K22" s="19"/>
+      <c r="K22" s="22"/>
       <c r="L22" s="13"/>
-      <c r="M22" s="19" t="s">
+      <c r="M22" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="N22" s="19"/>
+      <c r="N22" s="22"/>
       <c r="O22" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="74">
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="M22:N22"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A18:O18"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="K5:L5"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A6:O6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="K3:L3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="A5:B5"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="M11:O11"/>
@@ -2587,64 +2645,6 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D13:E13"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A6:O6"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="K3:L3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="K5:L5"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="A18:O18"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="G19:I19"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="D17:E17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -2665,11 +2665,10 @@
   <dimension ref="A1:E400"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
     <col min="2" max="2" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" style="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.28515625" style="16" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.5703125" style="18" customWidth="1"/>
+    <col min="3" max="4" width="20.7109375" style="16" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>